<commit_message>
Elimina duplicados de siete departamentos y actualiza mapas
Retira 37 registros repetidos y conserva intactos los seis departamentos excluidos. Publica solo esta depuracion, sin incorporar las actualizaciones locales pendientes de La Paz y La Libertad.
</commit_message>
<xml_diff>
--- a/data/por_departamento/Chalatenango/establecimientos_salud.xlsx
+++ b/data/por_departamento/Chalatenango/establecimientos_salud.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Establecimientos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Establecimientos'!$A$1:$AA$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Establecimientos'!$A$1:$AA$25</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA28"/>
+  <dimension ref="A1:AA25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1568,42 +1568,42 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>geofabrik-way-576913014</t>
+          <t>hot-way-765705663</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>geofabrik</t>
+          <t>hot</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>way/576913014</t>
+          <t>way/765705663</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Unidad de Salud</t>
+          <t>Unidad de Salud - La Palma</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Clínica</t>
+          <t>Hospital</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>clinica</t>
+          <t>hospital</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Predio</t>
+          <t>Polígono</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>predio</t>
+          <t>poligono</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1613,7 +1613,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Tejutla</t>
+          <t>La Palma</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1621,6 +1621,21 @@
           <t>Central</t>
         </is>
       </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>Medicina general</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>clinic</t>
+        </is>
+      </c>
       <c r="T12" t="inlineStr">
         <is>
           <t>Polygon</t>
@@ -1628,17 +1643,17 @@
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>14.1694194</t>
+          <t>14.31981955</t>
         </is>
       </c>
       <c r="W12" t="inlineStr">
         <is>
-          <t>-89.10106828</t>
+          <t>-89.17501211</t>
         </is>
       </c>
       <c r="X12" t="inlineStr">
@@ -1648,59 +1663,59 @@
       </c>
       <c r="Y12" t="inlineStr">
         <is>
-          <t>POLYGON ((-89.1012013 14.1693071, -89.1011872 14.1694974, -89.1011119 14.1694922, -89.1011068 14.1695618, -89.1009489 14.1695508, -89.1009681 14.1692908, -89.1012013 14.1693071))</t>
+          <t>POLYGON ((-89.1751896 14.3199335, -89.1751762 14.3196968, -89.1748272 14.3197046, -89.1748568 14.3199439, -89.1750393 14.3199413, -89.1751896 14.3199335))</t>
         </is>
       </c>
       <c r="Z12" t="inlineStr">
         <is>
-          <t>https://www.openstreetmap.org/way/576913014</t>
+          <t>https://www.openstreetmap.org/way/765705663</t>
         </is>
       </c>
       <c r="AA12" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=14.1694194,-89.10106828</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=14.31981955,-89.17501211</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>geofabrik-node-5879973979</t>
+          <t>hot-way-549827735</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>geofabrik</t>
+          <t>hot</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>node/5879973979</t>
+          <t>way/549827735</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Unidad de Salúd</t>
+          <t>Unidad de Salud Concepción Quezaltepeque</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Clínica</t>
+          <t>Hospital</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>clinica</t>
+          <t>hospital</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Punto</t>
+          <t>Polígono</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>punto</t>
+          <t>poligono</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1710,7 +1725,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>San Francisco Lempa</t>
+          <t>Concepción Quezaltepeque</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1718,51 +1733,71 @@
           <t>Central</t>
         </is>
       </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Concepción Quezaltepeque</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>Medicina general, Emergencia</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>Point</t>
+          <t>Polygon</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>13.973302</t>
+          <t>14.08466178</t>
         </is>
       </c>
       <c r="W13" t="inlineStr">
         <is>
-          <t>-88.9990673</t>
+          <t>-88.9637375</t>
         </is>
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>coordenada_original</t>
+          <t>centroide_area</t>
         </is>
       </c>
       <c r="Y13" t="inlineStr">
         <is>
-          <t>POINT (-88.9990673 13.973302)</t>
+          <t>POLYGON ((-88.9637121 14.0843626, -88.9633783 14.0846636, -88.9637885 14.0849673, -88.9640826 14.0846464, -88.9637121 14.0843626))</t>
         </is>
       </c>
       <c r="Z13" t="inlineStr">
         <is>
-          <t>https://www.openstreetmap.org/node/5879973979</t>
+          <t>https://www.openstreetmap.org/way/549827735</t>
         </is>
       </c>
       <c r="AA13" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=13.973302,-88.9990673</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=14.08466178,-88.9637375</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>hot-way-765705663</t>
+          <t>hot-node-8048941280</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1772,32 +1807,32 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>way/765705663</t>
+          <t>node/8048941280</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Unidad de Salud - La Palma</t>
+          <t>Clínica de Salud Digestiva San Antonio</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Hospital</t>
+          <t>Clínica</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>hospital</t>
+          <t>clinica</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Polígono</t>
+          <t>Punto</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>poligono</t>
+          <t>punto</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1817,64 +1852,54 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>Medicina general</t>
-        </is>
-      </c>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>hospital</t>
-        </is>
-      </c>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>clinic</t>
+          <t>Gastroenterología</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>Polygon</t>
+          <t>Point</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>14.31981955</t>
+          <t>14.3171692</t>
         </is>
       </c>
       <c r="W14" t="inlineStr">
         <is>
-          <t>-89.17501211</t>
+          <t>-89.1712624</t>
         </is>
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>centroide_area</t>
+          <t>coordenada_original</t>
         </is>
       </c>
       <c r="Y14" t="inlineStr">
         <is>
-          <t>POLYGON ((-89.1751896 14.3199335, -89.1751762 14.3196968, -89.1748272 14.3197046, -89.1748568 14.3199439, -89.1750393 14.3199413, -89.1751896 14.3199335))</t>
+          <t>POINT (-89.1712624 14.3171692)</t>
         </is>
       </c>
       <c r="Z14" t="inlineStr">
         <is>
-          <t>https://www.openstreetmap.org/way/765705663</t>
+          <t>https://www.openstreetmap.org/node/8048941280</t>
         </is>
       </c>
       <c r="AA14" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=14.31981955,-89.17501211</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=14.3171692,-89.1712624</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>hot-way-549827735</t>
+          <t>hot-node-6775076986</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1884,12 +1909,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>way/549827735</t>
+          <t>node/6775076986</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Unidad de Salud Concepción Quezaltepeque</t>
+          <t>Centro Médico La Palma</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1904,12 +1929,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Polígono</t>
+          <t>Punto</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>poligono</t>
+          <t>punto</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1919,7 +1944,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Concepción Quezaltepeque</t>
+          <t>La Palma</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1927,71 +1952,51 @@
           <t>Central</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>Concepción Quezaltepeque</t>
-        </is>
-      </c>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>Medicina general, Emergencia</t>
-        </is>
-      </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>hospital</t>
-        </is>
-      </c>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t>hospital</t>
-        </is>
-      </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>Polygon</t>
+          <t>Point</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>14.08466178</t>
+          <t>14.3181843</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>-88.9637375</t>
+          <t>-89.1714217</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>centroide_area</t>
+          <t>coordenada_original</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>POLYGON ((-88.9637121 14.0843626, -88.9633783 14.0846636, -88.9637885 14.0849673, -88.9640826 14.0846464, -88.9637121 14.0843626))</t>
+          <t>POINT (-89.1714217 14.3181843)</t>
         </is>
       </c>
       <c r="Z15" t="inlineStr">
         <is>
-          <t>https://www.openstreetmap.org/way/549827735</t>
+          <t>https://www.openstreetmap.org/node/6775076986</t>
         </is>
       </c>
       <c r="AA15" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=14.08466178,-88.9637375</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=14.3181843,-89.1714217</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>hot-way-576913014</t>
+          <t>hot-node-6777940386</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2001,12 +2006,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>way/576913014</t>
+          <t>node/6777940386</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Unidad de Salud</t>
+          <t>Granadilla La Palma</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -2021,12 +2026,12 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Polígono</t>
+          <t>Punto</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>poligono</t>
+          <t>punto</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -2036,7 +2041,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Tejutla</t>
+          <t>La Palma</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -2044,56 +2049,51 @@
           <t>Central</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>Santo Tomas Tejutla</t>
-        </is>
-      </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>Polygon</t>
+          <t>Point</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>14.1694194</t>
+          <t>14.3560439</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>-89.10106828</t>
+          <t>-89.0920045</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>centroide_area</t>
+          <t>coordenada_original</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>POLYGON ((-89.1009681 14.1692908, -89.1009489 14.1695508, -89.1011068 14.1695618, -89.1011119 14.1694922, -89.1011872 14.1694974, -89.1012013 14.1693071, -89.1009681 14.1692908))</t>
+          <t>POINT (-89.0920045 14.3560439)</t>
         </is>
       </c>
       <c r="Z16" t="inlineStr">
         <is>
-          <t>https://www.openstreetmap.org/way/576913014</t>
+          <t>https://www.openstreetmap.org/node/6777940386</t>
         </is>
       </c>
       <c r="AA16" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=14.1694194,-89.10106828</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=14.3560439,-89.0920045</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>hot-node-8048941280</t>
+          <t>hot-node-11461321169</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2103,12 +2103,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>node/8048941280</t>
+          <t>node/11461321169</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Clínica de Salud Digestiva San Antonio</t>
+          <t>Sin nombre</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -2138,7 +2138,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>La Palma</t>
+          <t>Chalatenango</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -2146,11 +2146,6 @@
           <t>Central</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>Gastroenterología</t>
-        </is>
-      </c>
       <c r="T17" t="inlineStr">
         <is>
           <t>Point</t>
@@ -2163,12 +2158,12 @@
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>14.3171692</t>
+          <t>14.0399619</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>-89.1712624</t>
+          <t>-88.9349105</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
@@ -2178,24 +2173,24 @@
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>POINT (-89.1712624 14.3171692)</t>
+          <t>POINT (-88.9349105 14.0399619)</t>
         </is>
       </c>
       <c r="Z17" t="inlineStr">
         <is>
-          <t>https://www.openstreetmap.org/node/8048941280</t>
+          <t>https://www.openstreetmap.org/node/11461321169</t>
         </is>
       </c>
       <c r="AA17" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=14.3171692,-89.1712624</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=14.0399619,-88.9349105</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>hot-node-6775076986</t>
+          <t>hot-node-11474266869</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2205,22 +2200,22 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>node/6775076986</t>
+          <t>node/11474266869</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Centro Médico La Palma</t>
+          <t>Clínica médica Casa de la Salud</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Hospital</t>
+          <t>Clínica</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>hospital</t>
+          <t>clinica</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -2240,7 +2235,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>La Palma</t>
+          <t>Chalatenango</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -2260,12 +2255,12 @@
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>14.3181843</t>
+          <t>14.039939</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>-89.1714217</t>
+          <t>-88.9349275</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
@@ -2275,24 +2270,24 @@
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>POINT (-89.1714217 14.3181843)</t>
+          <t>POINT (-88.9349275 14.039939)</t>
         </is>
       </c>
       <c r="Z18" t="inlineStr">
         <is>
-          <t>https://www.openstreetmap.org/node/6775076986</t>
+          <t>https://www.openstreetmap.org/node/11474266869</t>
         </is>
       </c>
       <c r="AA18" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=14.3181843,-89.1714217</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=14.039939,-88.9349275</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>hot-node-6777940386</t>
+          <t>hot-node-11483565869</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2302,12 +2297,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>node/6777940386</t>
+          <t>node/11483565869</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Granadilla La Palma</t>
+          <t>Clínica de Rayos-X, Chalatenango.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -2337,7 +2332,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>La Palma</t>
+          <t>Chalatenango</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -2357,12 +2352,12 @@
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>14.3560439</t>
+          <t>14.0399244</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>-89.0920045</t>
+          <t>-88.934849</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
@@ -2372,24 +2367,24 @@
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>POINT (-89.0920045 14.3560439)</t>
+          <t>POINT (-88.934849 14.0399244)</t>
         </is>
       </c>
       <c r="Z19" t="inlineStr">
         <is>
-          <t>https://www.openstreetmap.org/node/6777940386</t>
+          <t>https://www.openstreetmap.org/node/11483565869</t>
         </is>
       </c>
       <c r="AA19" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=14.3560439,-89.0920045</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=14.0399244,-88.934849</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>hot-node-11461321169</t>
+          <t>hot-node-3794782914</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2399,22 +2394,22 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>node/11461321169</t>
+          <t>node/3794782914</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Sin nombre</t>
+          <t>Unidad de Salud - San Miguel de Mercedes</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Clínica</t>
+          <t>Hospital</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>clinica</t>
+          <t>hospital</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -2434,7 +2429,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Chalatenango</t>
+          <t>San Miguel de Mercedes</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -2454,12 +2449,12 @@
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>14.0399619</t>
+          <t>14.0136776</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>-88.9349105</t>
+          <t>-88.9419111</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
@@ -2469,24 +2464,24 @@
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>POINT (-88.9349105 14.0399619)</t>
+          <t>POINT (-88.9419111 14.0136776)</t>
         </is>
       </c>
       <c r="Z20" t="inlineStr">
         <is>
-          <t>https://www.openstreetmap.org/node/11461321169</t>
+          <t>https://www.openstreetmap.org/node/3794782914</t>
         </is>
       </c>
       <c r="AA20" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=14.0399619,-88.9349105</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=14.0136776,-88.9419111</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>hot-node-11474266869</t>
+          <t>hot-node-4904550746</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2496,12 +2491,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>node/11474266869</t>
+          <t>node/4904550746</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Clínica médica Casa de la Salud</t>
+          <t>Centro Medico La Esperanza</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2531,7 +2526,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Chalatenango</t>
+          <t>Nueva Concepción</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -2551,12 +2546,12 @@
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>14.039939</t>
+          <t>14.1273057</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>-88.9349275</t>
+          <t>-89.2944363</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
@@ -2566,24 +2561,24 @@
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>POINT (-88.9349275 14.039939)</t>
+          <t>POINT (-89.2944363 14.1273057)</t>
         </is>
       </c>
       <c r="Z21" t="inlineStr">
         <is>
-          <t>https://www.openstreetmap.org/node/11474266869</t>
+          <t>https://www.openstreetmap.org/node/4904550746</t>
         </is>
       </c>
       <c r="AA21" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=14.039939,-88.9349275</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=14.1273057,-89.2944363</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>hot-node-11483565869</t>
+          <t>hot-node-4904550747</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2593,12 +2588,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>node/11483565869</t>
+          <t>node/4904550747</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Clínica de Rayos-X, Chalatenango.</t>
+          <t>Clínica de Especialidades Medico Quirurjico Shalom</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2628,7 +2623,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Chalatenango</t>
+          <t>Nueva Concepción</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -2648,12 +2643,12 @@
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>14.0399244</t>
+          <t>14.1267391</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>-88.934849</t>
+          <t>-89.2928713</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
@@ -2663,24 +2658,24 @@
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>POINT (-88.934849 14.0399244)</t>
+          <t>POINT (-89.2928713 14.1267391)</t>
         </is>
       </c>
       <c r="Z22" t="inlineStr">
         <is>
-          <t>https://www.openstreetmap.org/node/11483565869</t>
+          <t>https://www.openstreetmap.org/node/4904550747</t>
         </is>
       </c>
       <c r="AA22" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=14.0399244,-88.934849</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=14.1267391,-89.2928713</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>hot-node-3794782914</t>
+          <t>hot-node-4904550745</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2690,22 +2685,22 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>node/3794782914</t>
+          <t>node/4904550745</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Unidad de Salud - San Miguel de Mercedes</t>
+          <t>Clínica Medica Ultra Sonografica</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Hospital</t>
+          <t>Clínica</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>hospital</t>
+          <t>clinica</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2725,7 +2720,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>San Miguel de Mercedes</t>
+          <t>Nueva Concepción</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -2745,12 +2740,12 @@
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>14.0136776</t>
+          <t>14.1265882</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>-88.9419111</t>
+          <t>-89.2912327</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
@@ -2760,24 +2755,24 @@
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>POINT (-88.9419111 14.0136776)</t>
+          <t>POINT (-89.2912327 14.1265882)</t>
         </is>
       </c>
       <c r="Z23" t="inlineStr">
         <is>
-          <t>https://www.openstreetmap.org/node/3794782914</t>
+          <t>https://www.openstreetmap.org/node/4904550745</t>
         </is>
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=14.0136776,-88.9419111</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=14.1265882,-89.2912327</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>hot-node-4904550746</t>
+          <t>hot-node-5879973979</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2787,12 +2782,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>node/4904550746</t>
+          <t>node/5879973979</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Centro Medico La Esperanza</t>
+          <t>Unidad de Salúd</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2822,7 +2817,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Nueva Concepción</t>
+          <t>Azacualpa</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2830,6 +2825,11 @@
           <t>Central</t>
         </is>
       </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>San Francisco Lempa</t>
+        </is>
+      </c>
       <c r="T24" t="inlineStr">
         <is>
           <t>Point</t>
@@ -2842,12 +2842,12 @@
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>14.1273057</t>
+          <t>13.973302</t>
         </is>
       </c>
       <c r="W24" t="inlineStr">
         <is>
-          <t>-89.2944363</t>
+          <t>-88.9990673</t>
         </is>
       </c>
       <c r="X24" t="inlineStr">
@@ -2857,24 +2857,24 @@
       </c>
       <c r="Y24" t="inlineStr">
         <is>
-          <t>POINT (-89.2944363 14.1273057)</t>
+          <t>POINT (-88.9990673 13.973302)</t>
         </is>
       </c>
       <c r="Z24" t="inlineStr">
         <is>
-          <t>https://www.openstreetmap.org/node/4904550746</t>
+          <t>https://www.openstreetmap.org/node/5879973979</t>
         </is>
       </c>
       <c r="AA24" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=14.1273057,-89.2944363</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=13.973302,-88.9990673</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>hot-node-4904550747</t>
+          <t>hot-node-11812898625</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2884,22 +2884,22 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>node/4904550747</t>
+          <t>node/11812898625</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Clínica de Especialidades Medico Quirurjico Shalom</t>
+          <t>Unidad Comunitaria de Salud Familiar de El Paraíso</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Clínica</t>
+          <t>Consultorio</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>clinica</t>
+          <t>consultorio</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2919,7 +2919,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Nueva Concepción</t>
+          <t>El Paraíso</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2939,12 +2939,12 @@
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>14.1267391</t>
+          <t>14.1090348</t>
         </is>
       </c>
       <c r="W25" t="inlineStr">
         <is>
-          <t>-89.2928713</t>
+          <t>-89.0682761</t>
         </is>
       </c>
       <c r="X25" t="inlineStr">
@@ -2954,318 +2954,22 @@
       </c>
       <c r="Y25" t="inlineStr">
         <is>
-          <t>POINT (-89.2928713 14.1267391)</t>
+          <t>POINT (-89.0682761 14.1090348)</t>
         </is>
       </c>
       <c r="Z25" t="inlineStr">
         <is>
-          <t>https://www.openstreetmap.org/node/4904550747</t>
+          <t>https://www.openstreetmap.org/node/11812898625</t>
         </is>
       </c>
       <c r="AA25" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=14.1267391,-89.2928713</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>hot-node-4904550745</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>hot</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>node/4904550745</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Clínica Medica Ultra Sonografica</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>Clínica</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>clinica</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>Punto</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>punto</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>Chalatenango</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>Nueva Concepción</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>Central</t>
-        </is>
-      </c>
-      <c r="T26" t="inlineStr">
-        <is>
-          <t>Point</t>
-        </is>
-      </c>
-      <c r="U26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="V26" t="inlineStr">
-        <is>
-          <t>14.1265882</t>
-        </is>
-      </c>
-      <c r="W26" t="inlineStr">
-        <is>
-          <t>-89.2912327</t>
-        </is>
-      </c>
-      <c r="X26" t="inlineStr">
-        <is>
-          <t>coordenada_original</t>
-        </is>
-      </c>
-      <c r="Y26" t="inlineStr">
-        <is>
-          <t>POINT (-89.2912327 14.1265882)</t>
-        </is>
-      </c>
-      <c r="Z26" t="inlineStr">
-        <is>
-          <t>https://www.openstreetmap.org/node/4904550745</t>
-        </is>
-      </c>
-      <c r="AA26" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=14.1265882,-89.2912327</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>hot-node-5879973979</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>hot</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>node/5879973979</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Unidad de Salúd</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>Clínica</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>clinica</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>Punto</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>punto</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>Chalatenango</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>Azacualpa</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>Central</t>
-        </is>
-      </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>San Francisco Lempa</t>
-        </is>
-      </c>
-      <c r="T27" t="inlineStr">
-        <is>
-          <t>Point</t>
-        </is>
-      </c>
-      <c r="U27" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="V27" t="inlineStr">
-        <is>
-          <t>13.973302</t>
-        </is>
-      </c>
-      <c r="W27" t="inlineStr">
-        <is>
-          <t>-88.9990673</t>
-        </is>
-      </c>
-      <c r="X27" t="inlineStr">
-        <is>
-          <t>coordenada_original</t>
-        </is>
-      </c>
-      <c r="Y27" t="inlineStr">
-        <is>
-          <t>POINT (-88.9990673 13.973302)</t>
-        </is>
-      </c>
-      <c r="Z27" t="inlineStr">
-        <is>
-          <t>https://www.openstreetmap.org/node/5879973979</t>
-        </is>
-      </c>
-      <c r="AA27" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=13.973302,-88.9990673</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>hot-node-11812898625</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>hot</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>node/11812898625</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Unidad Comunitaria de Salud Familiar de El Paraíso</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>Consultorio</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>consultorio</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>Punto</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>punto</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>Chalatenango</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>El Paraíso</t>
-        </is>
-      </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>Central</t>
-        </is>
-      </c>
-      <c r="T28" t="inlineStr">
-        <is>
-          <t>Point</t>
-        </is>
-      </c>
-      <c r="U28" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="V28" t="inlineStr">
-        <is>
-          <t>14.1090348</t>
-        </is>
-      </c>
-      <c r="W28" t="inlineStr">
-        <is>
-          <t>-89.0682761</t>
-        </is>
-      </c>
-      <c r="X28" t="inlineStr">
-        <is>
-          <t>coordenada_original</t>
-        </is>
-      </c>
-      <c r="Y28" t="inlineStr">
-        <is>
-          <t>POINT (-89.0682761 14.1090348)</t>
-        </is>
-      </c>
-      <c r="Z28" t="inlineStr">
-        <is>
-          <t>https://www.openstreetmap.org/node/11812898625</t>
-        </is>
-      </c>
-      <c r="AA28" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=14.1090348,-89.0682761</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AA28"/>
+  <autoFilter ref="A1:AA25"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>